<commit_message>
feat(imports): skip deferred-card settlement lines to avoid double counting
CM/CIC current-account exports carry a monthly "RELEVE CARTE" aggregate
that settles a deferred-debit card. Its itemized detail lives on the card
statement sheets, so importing both double-counts spending. Skip the
aggregate (narrowly matched, never touching "PAIEMENT ... CARTE",
"RETRAIT DAB ... CARTE", fees, etc.) and keep the detail.

- AccountSheetDetector: CARD_SETTLEMENT_PATTERNS + card_settlement? filter
- fixture: add a RELEVE CARTE row + test it is skipped
- sheet-selection UI: note that aggregate card lines are auto-excluded

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/files/imports/sample_bank_export.xlsx
+++ b/test/fixtures/files/imports/sample_bank_export.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,20 +607,41 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
+        <v>46051</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46051</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>RELEVE CARTE</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B9" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>NOUVEAU TAUX</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E9" t="n">
         <v>0</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
@@ -795,7 +816,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A6:E8</t>
+          <t>A6:E9</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>

<commit_message>
Revert "feat(imports): skip deferred-card settlement lines to avoid double counting"
This reverts commit 7fc589857ba4551ed10dda81d6d5622843aad063.
</commit_message>
<xml_diff>
--- a/test/fixtures/files/imports/sample_bank_export.xlsx
+++ b/test/fixtures/files/imports/sample_bank_export.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,41 +607,20 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46051</v>
+        <v>46054</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46051</v>
+        <v>46054</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RELEVE CARTE</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>-100</v>
+          <t>NOUVEAU TAUX</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
       </c>
       <c r="G8" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46054</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>46054</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>NOUVEAU TAUX</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
@@ -816,7 +795,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A6:E9</t>
+          <t>A6:E8</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>